<commit_message>
Use goldpricez 21K prices for 14-28 October
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01C3cFR25ukD86hWgq7s1XGY
</commit_message>
<xml_diff>
--- a/data/markets.xlsx
+++ b/data/markets.xlsx
@@ -3585,7 +3585,7 @@
       <c r="D118" s="2" t="n"/>
       <c r="E118" s="2" t="n"/>
       <c r="F118" s="2" t="n">
-        <v>6129</v>
+        <v>6130.04</v>
       </c>
       <c r="G118" s="2" t="n">
         <v>4107.9</v>
@@ -3626,7 +3626,7 @@
       <c r="D119" s="2" t="n"/>
       <c r="E119" s="2" t="n"/>
       <c r="F119" s="2" t="n">
-        <v>6270</v>
+        <v>6269.6</v>
       </c>
       <c r="G119" s="2" t="n">
         <v>4170.1</v>
@@ -3663,7 +3663,7 @@
       <c r="D120" s="2" t="n"/>
       <c r="E120" s="2" t="n"/>
       <c r="F120" s="2" t="n">
-        <v>6263</v>
+        <v>6270.26</v>
       </c>
       <c r="G120" s="2" t="n">
         <v>4181.1</v>
@@ -3697,7 +3697,9 @@
       <c r="C121" s="2" t="n"/>
       <c r="D121" s="2" t="n"/>
       <c r="E121" s="2" t="n"/>
-      <c r="F121" s="2" t="n"/>
+      <c r="F121" s="2" t="n">
+        <v>6270.26</v>
+      </c>
       <c r="G121" s="2" t="n"/>
       <c r="H121" s="2" t="n"/>
       <c r="I121" s="2" t="n"/>
@@ -3726,7 +3728,9 @@
       </c>
       <c r="D122" s="2" t="n"/>
       <c r="E122" s="2" t="n"/>
-      <c r="F122" s="2" t="n"/>
+      <c r="F122" s="2" t="n">
+        <v>6281.98</v>
+      </c>
       <c r="G122" s="2" t="n"/>
       <c r="H122" s="2" t="n"/>
       <c r="I122" s="2" t="n">
@@ -3758,7 +3762,7 @@
       <c r="D123" s="2" t="n"/>
       <c r="E123" s="2" t="n"/>
       <c r="F123" s="2" t="n">
-        <v>6280</v>
+        <v>6283.2</v>
       </c>
       <c r="G123" s="2" t="n">
         <v>4160.1</v>
@@ -3799,7 +3803,7 @@
       <c r="D124" s="2" t="n"/>
       <c r="E124" s="2" t="n"/>
       <c r="F124" s="2" t="n">
-        <v>6324</v>
+        <v>6328.62</v>
       </c>
       <c r="G124" s="2" t="n">
         <v>4142.6</v>
@@ -3840,7 +3844,7 @@
       <c r="D125" s="2" t="n"/>
       <c r="E125" s="2" t="n"/>
       <c r="F125" s="2" t="n">
-        <v>6335</v>
+        <v>6335.61</v>
       </c>
       <c r="G125" s="2" t="n">
         <v>4150</v>
@@ -3881,7 +3885,7 @@
       <c r="D126" s="2" t="n"/>
       <c r="E126" s="2" t="n"/>
       <c r="F126" s="2" t="n">
-        <v>6261</v>
+        <v>6261.48</v>
       </c>
       <c r="G126" s="2" t="n">
         <v>4060.4</v>
@@ -3918,7 +3922,7 @@
       <c r="D127" s="2" t="n"/>
       <c r="E127" s="2" t="n"/>
       <c r="F127" s="2" t="n">
-        <v>6216</v>
+        <v>6217.01</v>
       </c>
       <c r="G127" s="2" t="n">
         <v>4007.9</v>
@@ -3952,7 +3956,9 @@
       <c r="C128" s="2" t="n"/>
       <c r="D128" s="2" t="n"/>
       <c r="E128" s="2" t="n"/>
-      <c r="F128" s="2" t="n"/>
+      <c r="F128" s="2" t="n">
+        <v>6217.01</v>
+      </c>
       <c r="G128" s="2" t="n"/>
       <c r="H128" s="2" t="n"/>
       <c r="I128" s="2" t="n"/>
@@ -3977,7 +3983,9 @@
       <c r="C129" s="2" t="n"/>
       <c r="D129" s="2" t="n"/>
       <c r="E129" s="2" t="n"/>
-      <c r="F129" s="2" t="n"/>
+      <c r="F129" s="2" t="n">
+        <v>6275.47</v>
+      </c>
       <c r="G129" s="2" t="n"/>
       <c r="H129" s="2" t="n"/>
       <c r="I129" s="2" t="n">
@@ -4009,7 +4017,7 @@
       <c r="D130" s="2" t="n"/>
       <c r="E130" s="2" t="n"/>
       <c r="F130" s="2" t="n">
-        <v>6359</v>
+        <v>6358.34</v>
       </c>
       <c r="G130" s="2" t="n">
         <v>4038.4</v>
@@ -4087,7 +4095,7 @@
       <c r="D132" s="2" t="n"/>
       <c r="E132" s="2" t="n"/>
       <c r="F132" s="2" t="n">
-        <v>6393</v>
+        <v>6410.65</v>
       </c>
       <c r="G132" s="2" t="n"/>
       <c r="H132" s="2" t="n"/>

</xml_diff>